<commit_message>
data reconstruction & report update
</commit_message>
<xml_diff>
--- a/aec/results/강남/feature_selection_report.xlsx
+++ b/aec/results/강남/feature_selection_report.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="상관계수_전체" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="상관계수_Top20" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="VIF_선택feature" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="TAMA_분포_성별" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="상관계수_전체" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="상관계수_Top20" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VIF_선택feature" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TAMA_분포_성별" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -479,34 +479,34 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>skewness</t>
+          <t>p25</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>-3.3129e-01</t>
+          <t>3.6644e-01</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>8.6009e-46</t>
+          <t>2.5306e-54</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>-3.3399e-01</t>
+          <t>3.6956e-01</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1.4808e-46</t>
+          <t>2.7359e-55</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>1738</v>
+        <v>1673</v>
       </c>
       <c r="H2" t="n">
-        <v>0.33129</v>
+        <v>0.36644</v>
       </c>
     </row>
     <row r="3">
@@ -515,34 +515,34 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>p25</t>
+          <t>p10</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>3.0930e-01</t>
+          <t>3.5776e-01</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>4.0245e-46</t>
+          <t>1.0943e-51</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>3.1692e-01</t>
+          <t>3.5255e-01</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>1.8684e-48</t>
+          <t>3.8373e-50</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H3" t="n">
-        <v>0.3093</v>
+        <v>0.35776</v>
       </c>
     </row>
     <row r="4">
@@ -551,34 +551,34 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>p10</t>
+          <t>CV</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3.0799e-01</t>
+          <t>-3.4903e-01</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>9.9720e-46</t>
+          <t>4.0679e-49</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>3.1347e-01</t>
+          <t>-3.5984e-01</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2.1750e-47</t>
+          <t>2.5995e-52</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H4" t="n">
-        <v>0.30799</v>
+        <v>0.34903</v>
       </c>
     </row>
     <row r="5">
@@ -592,29 +592,29 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3.0341e-01</t>
+          <t>3.4342e-01</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2.2993e-44</t>
+          <t>1.6487e-47</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2.7255e-01</t>
+          <t>3.2372e-01</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>8.3381e-36</t>
+          <t>4.0805e-42</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H5" t="n">
-        <v>0.30341</v>
+        <v>0.34342</v>
       </c>
     </row>
     <row r="6">
@@ -623,34 +623,34 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>AUC</t>
+          <t>skewness</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2.9834e-01</t>
+          <t>-3.4332e-01</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6.9312e-43</t>
+          <t>1.7578e-47</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>3.0392e-01</t>
+          <t>-3.2715e-01</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>1.6227e-44</t>
+          <t>5.0009e-43</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H6" t="n">
-        <v>0.29834</v>
+        <v>0.34332</v>
       </c>
     </row>
     <row r="7">
@@ -659,34 +659,34 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>peak_mean_height</t>
+          <t>kurtosis</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2.9743e-01</t>
+          <t>3.3102e-01</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1.6018e-35</t>
+          <t>4.5303e-44</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>3.2378e-01</t>
+          <t>3.8909e-01</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>3.9207e-42</t>
+          <t>1.3591e-61</t>
         </is>
       </c>
       <c r="G7" t="n">
         <v>1673</v>
       </c>
       <c r="H7" t="n">
-        <v>0.29743</v>
+        <v>0.33102</v>
       </c>
     </row>
     <row r="8">
@@ -695,34 +695,34 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>wavelet_cA_energy</t>
+          <t>AUC</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2.8136e-01</t>
+          <t>3.3086e-01</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.8634e-38</t>
+          <t>5.0127e-44</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2.4854e-01</t>
+          <t>3.4466e-01</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>7.1358e-30</t>
+          <t>7.3014e-48</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H8" t="n">
-        <v>0.28136</v>
+        <v>0.33086</v>
       </c>
     </row>
     <row r="9">
@@ -731,34 +731,34 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>kurtosis</t>
+          <t>median</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2.7751e-01</t>
+          <t>3.2903e-01</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>4.2214e-32</t>
+          <t>1.5664e-43</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3.9515e-01</t>
+          <t>3.3747e-01</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>4.8330e-66</t>
+          <t>7.7459e-46</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>1738</v>
+        <v>1673</v>
       </c>
       <c r="H9" t="n">
-        <v>0.27751</v>
+        <v>0.32903</v>
       </c>
     </row>
     <row r="10">
@@ -767,34 +767,34 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>p5</t>
+          <t>wavelet_cA_energy</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2.7029e-01</t>
+          <t>3.2281e-01</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>3.1972e-35</t>
+          <t>7.0719e-42</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2.7232e-01</t>
+          <t>2.9972e-01</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>9.5299e-36</t>
+          <t>4.5505e-36</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H10" t="n">
-        <v>0.27029</v>
+        <v>0.32281</v>
       </c>
     </row>
     <row r="11">
@@ -803,34 +803,34 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>median</t>
+          <t>p90_p10_ratio</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2.6759e-01</t>
+          <t>-3.1834e-01</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1.5694e-34</t>
+          <t>1.0327e-40</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2.7686e-01</t>
+          <t>-3.5191e-01</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>6.1348e-37</t>
+          <t>5.9040e-50</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H11" t="n">
-        <v>0.26759</v>
+        <v>0.31834</v>
       </c>
     </row>
     <row r="12">
@@ -839,34 +839,34 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>min</t>
+          <t>p5</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2.6597e-01</t>
+          <t>3.0393e-01</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>4.0645e-34</t>
+          <t>4.3413e-37</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2.7455e-01</t>
+          <t>2.9402e-01</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2.4949e-36</t>
+          <t>1.0259e-34</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H12" t="n">
-        <v>0.26597</v>
+        <v>0.30393</v>
       </c>
     </row>
     <row r="13">
@@ -875,34 +875,34 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>p90_p10_ratio</t>
+          <t>min</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>-2.6350e-01</t>
+          <t>2.9746e-01</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>1.6941e-33</t>
+          <t>1.5763e-35</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>-2.8949e-01</t>
+          <t>2.9885e-01</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2.2689e-40</t>
+          <t>7.3495e-36</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H13" t="n">
-        <v>0.2635</v>
+        <v>0.29746</v>
       </c>
     </row>
     <row r="14">
@@ -911,34 +911,34 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>peak_max_width</t>
+          <t>peak_mean_height</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2.6156e-01</t>
+          <t>2.9743e-01</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>1.4288e-27</t>
+          <t>1.6018e-35</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>3.0469e-01</t>
+          <t>3.2378e-01</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2.8193e-37</t>
+          <t>3.9207e-42</t>
         </is>
       </c>
       <c r="G14" t="n">
         <v>1673</v>
       </c>
       <c r="H14" t="n">
-        <v>0.26156</v>
+        <v>0.29743</v>
       </c>
     </row>
     <row r="15">
@@ -947,34 +947,34 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CV</t>
+          <t>AUC_normalized</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>-2.5882e-01</t>
+          <t>2.9738e-01</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2.4535e-32</t>
+          <t>1.6476e-35</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>-2.9598e-01</t>
+          <t>3.0680e-01</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>3.3202e-42</t>
+          <t>8.5343e-38</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H15" t="n">
-        <v>0.25882</v>
+        <v>0.29738</v>
       </c>
     </row>
     <row r="16">
@@ -983,34 +983,34 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>peak_max_height</t>
+          <t>mean</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2.4627e-01</t>
+          <t>2.9683e-01</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>1.5613e-24</t>
+          <t>2.2272e-35</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2.7520e-01</t>
+          <t>3.0620e-01</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>1.8682e-30</t>
+          <t>1.1995e-37</t>
         </is>
       </c>
       <c r="G16" t="n">
         <v>1673</v>
       </c>
       <c r="H16" t="n">
-        <v>0.24627</v>
+        <v>0.29683</v>
       </c>
     </row>
     <row r="17">
@@ -1019,34 +1019,34 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>AUC_normalized</t>
+          <t>IQR</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2.3893e-01</t>
+          <t>-2.6372e-01</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1.1413e-27</t>
+          <t>5.1269e-28</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2.5128e-01</t>
+          <t>-2.8742e-01</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>1.6169e-30</t>
+          <t>3.4962e-33</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H17" t="n">
-        <v>0.23893</v>
+        <v>0.26372</v>
       </c>
     </row>
     <row r="18">
@@ -1055,34 +1055,34 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>mean</t>
+          <t>peak_max_width</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2.3835e-01</t>
+          <t>2.6156e-01</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>1.5393e-27</t>
+          <t>1.4288e-27</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2.4982e-01</t>
+          <t>3.0469e-01</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>3.5831e-30</t>
+          <t>2.8193e-37</t>
         </is>
       </c>
       <c r="G18" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H18" t="n">
-        <v>0.23835</v>
+        <v>0.26156</v>
       </c>
     </row>
     <row r="19">
@@ -1091,34 +1091,34 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>peak_mean_width</t>
+          <t>peak_max_height</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2.3665e-01</t>
+          <t>2.4627e-01</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1.0010e-22</t>
+          <t>1.5613e-24</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2.4913e-01</t>
+          <t>2.7520e-01</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>4.3631e-25</t>
+          <t>1.8682e-30</t>
         </is>
       </c>
       <c r="G19" t="n">
         <v>1673</v>
       </c>
       <c r="H19" t="n">
-        <v>0.23665</v>
+        <v>0.24627</v>
       </c>
     </row>
     <row r="20">
@@ -1127,34 +1127,34 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>IQR</t>
+          <t>dominant_freq</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>-2.2228e-01</t>
+          <t>2.4549e-01</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>4.4729e-24</t>
+          <t>2.1957e-24</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>-2.4286e-01</t>
+          <t>1.9218e-01</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>1.4700e-28</t>
+          <t>2.2173e-15</t>
         </is>
       </c>
       <c r="G20" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H20" t="n">
-        <v>0.22228</v>
+        <v>0.24549</v>
       </c>
     </row>
     <row r="21">
@@ -1163,34 +1163,34 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>signal_length</t>
+          <t>peak_mean_width</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>1.9536e-01</t>
+          <t>2.3665e-01</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>7.3748e-19</t>
+          <t>1.0010e-22</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2.4338e-01</t>
+          <t>2.4913e-01</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>1.1199e-28</t>
+          <t>4.3631e-25</t>
         </is>
       </c>
       <c r="G21" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H21" t="n">
-        <v>0.19536</v>
+        <v>0.23665</v>
       </c>
     </row>
     <row r="22">
@@ -1204,29 +1204,29 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-1.7476e-01</t>
+          <t>-2.1564e-01</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2.4063e-15</t>
+          <t>4.7200e-19</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-1.9424e-01</t>
+          <t>-2.2245e-01</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>1.1703e-18</t>
+          <t>3.3416e-20</t>
         </is>
       </c>
       <c r="G22" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H22" t="n">
-        <v>0.17476</v>
+        <v>0.21564</v>
       </c>
     </row>
     <row r="23">
@@ -1235,34 +1235,34 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>peak_main_pos</t>
+          <t>p75</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1.6366e-01</t>
+          <t>2.1010e-01</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.6423e-11</t>
+          <t>3.8114e-18</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.5743e-01</t>
+          <t>2.2124e-01</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>9.4834e-11</t>
+          <t>5.3745e-20</t>
         </is>
       </c>
       <c r="G23" t="n">
         <v>1673</v>
       </c>
       <c r="H23" t="n">
-        <v>0.16366</v>
+        <v>0.2101</v>
       </c>
     </row>
     <row r="24">
@@ -1271,34 +1271,34 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>peak_std_height</t>
+          <t>zero_crossing_rate</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>-1.6092e-01</t>
+          <t>1.9039e-01</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>3.5898e-11</t>
+          <t>4.0501e-15</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>-1.0885e-01</t>
+          <t>2.9350e-01</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>8.1212e-06</t>
+          <t>1.3639e-34</t>
         </is>
       </c>
       <c r="G24" t="n">
         <v>1673</v>
       </c>
       <c r="H24" t="n">
-        <v>0.16092</v>
+        <v>0.19039</v>
       </c>
     </row>
     <row r="25">
@@ -1307,34 +1307,34 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>p75</t>
+          <t>p90</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>1.6027e-01</t>
+          <t>1.8938e-01</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>4.0749e-13</t>
+          <t>5.6611e-15</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.6802e-01</t>
+          <t>2.0398e-01</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2.7747e-14</t>
+          <t>3.5787e-17</t>
         </is>
       </c>
       <c r="G25" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H25" t="n">
-        <v>0.16027</v>
+        <v>0.18938</v>
       </c>
     </row>
     <row r="26">
@@ -1343,34 +1343,34 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>first_high_pos</t>
+          <t>max</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>1.5380e-01</t>
+          <t>1.8931e-01</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>3.4926e-12</t>
+          <t>5.8005e-15</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2.5916e-02</t>
+          <t>2.1072e-01</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2.4385e-01</t>
+          <t>3.0306e-18</t>
         </is>
       </c>
       <c r="G26" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H26" t="n">
-        <v>0.1538</v>
+        <v>0.18931</v>
       </c>
     </row>
     <row r="27">
@@ -1379,34 +1379,34 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>zero_crossing_rate</t>
+          <t>p95</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>1.5149e-01</t>
+          <t>1.8782e-01</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>7.3461e-12</t>
+          <t>9.5165e-15</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1.8739e-01</t>
+          <t>2.0471e-01</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>1.8887e-17</t>
+          <t>2.7569e-17</t>
         </is>
       </c>
       <c r="G27" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H27" t="n">
-        <v>0.15149</v>
+        <v>0.18782</v>
       </c>
     </row>
     <row r="28">
@@ -1415,34 +1415,34 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>p90</t>
+          <t>first_high_pos</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>1.4123e-01</t>
+          <t>1.8460e-01</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>1.7515e-10</t>
+          <t>2.7342e-14</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1.5125e-01</t>
+          <t>7.8323e-02</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>7.9234e-12</t>
+          <t>1.3453e-03</t>
         </is>
       </c>
       <c r="G28" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H28" t="n">
-        <v>0.14123</v>
+        <v>0.1846</v>
       </c>
     </row>
     <row r="29">
@@ -1451,34 +1451,34 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>p95</t>
+          <t>signal_length</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>1.3916e-01</t>
+          <t>1.7483e-01</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>3.2324e-10</t>
+          <t>5.9710e-13</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.5113e-01</t>
+          <t>2.5069e-01</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>8.2397e-12</t>
+          <t>2.1622e-25</t>
         </is>
       </c>
       <c r="G29" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H29" t="n">
-        <v>0.13916</v>
+        <v>0.17483</v>
       </c>
     </row>
     <row r="30">
@@ -1487,34 +1487,34 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>max</t>
+          <t>peak_main_pos</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>1.3899e-01</t>
+          <t>1.6366e-01</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>3.3943e-10</t>
+          <t>1.6423e-11</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1.5456e-01</t>
+          <t>1.5743e-01</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2.7285e-12</t>
+          <t>9.4834e-11</t>
         </is>
       </c>
       <c r="G30" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H30" t="n">
-        <v>0.13899</v>
+        <v>0.16366</v>
       </c>
     </row>
     <row r="31">
@@ -1523,34 +1523,34 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>fft_mag_max</t>
+          <t>peak_std_height</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>-1.3615e-01</t>
+          <t>-1.6092e-01</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>7.7337e-10</t>
+          <t>3.5898e-11</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>-1.6703e-01</t>
+          <t>-1.0885e-01</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>3.9403e-14</t>
+          <t>8.1212e-06</t>
         </is>
       </c>
       <c r="G31" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H31" t="n">
-        <v>0.13615</v>
+        <v>0.16092</v>
       </c>
     </row>
     <row r="32">
@@ -1559,34 +1559,34 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>std</t>
+          <t>fft_mag_max</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>-1.2235e-01</t>
+          <t>-1.5607e-01</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>3.3599e-08</t>
+          <t>1.3781e-10</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>-1.3676e-01</t>
+          <t>-1.8687e-01</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>6.4999e-10</t>
+          <t>1.3033e-14</t>
         </is>
       </c>
       <c r="G32" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H32" t="n">
-        <v>0.12235</v>
+        <v>0.15607</v>
       </c>
     </row>
     <row r="33">
@@ -1595,34 +1595,34 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>RMSE</t>
+          <t>slope_min</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>-1.2220e-01</t>
+          <t>-1.5390e-01</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>3.4854e-08</t>
+          <t>2.4877e-10</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>-1.3663e-01</t>
+          <t>-1.2238e-01</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>6.7354e-10</t>
+          <t>5.1453e-07</t>
         </is>
       </c>
       <c r="G33" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H33" t="n">
-        <v>0.1222</v>
+        <v>0.1539</v>
       </c>
     </row>
     <row r="34">
@@ -1631,34 +1631,34 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>slope_mean</t>
+          <t>spectral_centroid</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>1.1214e-01</t>
+          <t>1.4823e-01</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>4.2403e-07</t>
+          <t>1.1155e-09</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>1.1672e-01</t>
+          <t>1.9101e-01</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>1.3940e-07</t>
+          <t>3.2837e-15</t>
         </is>
       </c>
       <c r="G34" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H34" t="n">
-        <v>0.11214</v>
+        <v>0.14823</v>
       </c>
     </row>
     <row r="35">
@@ -1667,34 +1667,34 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>slope_min</t>
+          <t>std</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>-1.0848e-01</t>
+          <t>-1.4693e-01</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>9.9846e-07</t>
+          <t>1.5576e-09</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>-6.5257e-02</t>
+          <t>-1.4380e-01</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>3.3121e-03</t>
+          <t>3.4619e-09</t>
         </is>
       </c>
       <c r="G35" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H35" t="n">
-        <v>0.10848</v>
+        <v>0.14693</v>
       </c>
     </row>
     <row r="36">
@@ -1703,34 +1703,34 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>wavelet_cA_std</t>
+          <t>RMSE</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>-1.0654e-01</t>
+          <t>-1.4673e-01</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>1.5575e-06</t>
+          <t>1.6439e-09</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>-1.1839e-01</t>
+          <t>-1.4362e-01</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>9.1969e-08</t>
+          <t>3.6199e-09</t>
         </is>
       </c>
       <c r="G36" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H36" t="n">
-        <v>0.10654</v>
+        <v>0.14673</v>
       </c>
     </row>
     <row r="37">
@@ -1739,34 +1739,34 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>fft_mag_std</t>
+          <t>slope_std</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>-9.9994e-02</t>
+          <t>1.3741e-01</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>6.5710e-06</t>
+          <t>1.6718e-08</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>-1.2001e-01</t>
+          <t>1.5751e-01</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>6.1204e-08</t>
+          <t>9.2840e-11</t>
         </is>
       </c>
       <c r="G37" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H37" t="n">
-        <v>0.099994</v>
+        <v>0.13741</v>
       </c>
     </row>
     <row r="38">
@@ -1775,34 +1775,34 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>slope_std</t>
+          <t>wavelet_cA_std</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>8.2173e-02</t>
+          <t>-1.2258e-01</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>2.1487e-04</t>
+          <t>4.9337e-07</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>8.9673e-02</t>
+          <t>-1.1753e-01</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>5.3469e-05</t>
+          <t>1.4327e-06</t>
         </is>
       </c>
       <c r="G38" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H38" t="n">
-        <v>0.082173</v>
+        <v>0.12258</v>
       </c>
     </row>
     <row r="39">
@@ -1811,34 +1811,34 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>peak_last_pos</t>
+          <t>slope_mean</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>7.6832e-02</t>
+          <t>1.1722e-01</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>1.6614e-03</t>
+          <t>1.5289e-06</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>-7.9049e-02</t>
+          <t>1.0847e-01</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>1.2124e-03</t>
+          <t>8.7259e-06</t>
         </is>
       </c>
       <c r="G39" t="n">
         <v>1673</v>
       </c>
       <c r="H39" t="n">
-        <v>0.076832</v>
+        <v>0.11722</v>
       </c>
     </row>
     <row r="40">
@@ -1847,34 +1847,34 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>peak_first_pos</t>
+          <t>fft_mag_std</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>7.4971e-02</t>
+          <t>-1.1269e-01</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>2.1513e-03</t>
+          <t>3.8286e-06</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>7.5897e-02</t>
+          <t>-1.2387e-01</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>1.8930e-03</t>
+          <t>3.7263e-07</t>
         </is>
       </c>
       <c r="G40" t="n">
         <v>1673</v>
       </c>
       <c r="H40" t="n">
-        <v>0.074971</v>
+        <v>0.11269</v>
       </c>
     </row>
     <row r="41">
@@ -1883,34 +1883,34 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>valley_count</t>
+          <t>spectral_rolloff</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>6.6953e-02</t>
+          <t>1.0681e-01</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>2.5813e-03</t>
+          <t>1.1972e-05</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>9.3704e-02</t>
+          <t>1.6081e-01</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2.4179e-05</t>
+          <t>3.6970e-11</t>
         </is>
       </c>
       <c r="G41" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H41" t="n">
-        <v>0.066953</v>
+        <v>0.10681</v>
       </c>
     </row>
     <row r="42">
@@ -1919,34 +1919,34 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>dominant_freq</t>
+          <t>wavelet_cD1_energy</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>6.6671e-02</t>
+          <t>8.4318e-02</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>2.6917e-03</t>
+          <t>5.5571e-04</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>1.5348e-01</t>
+          <t>7.6399e-02</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>3.8679e-12</t>
+          <t>1.7653e-03</t>
         </is>
       </c>
       <c r="G42" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H42" t="n">
-        <v>0.06667099999999999</v>
+        <v>0.084318</v>
       </c>
     </row>
     <row r="43">
@@ -1955,34 +1955,34 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>wavelet_cD1_energy</t>
+          <t>valley_count</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>6.3089e-02</t>
+          <t>8.2693e-02</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>4.5204e-03</t>
+          <t>7.1020e-04</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>3.3006e-02</t>
+          <t>1.3548e-01</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>1.3770e-01</t>
+          <t>2.6495e-08</t>
         </is>
       </c>
       <c r="G43" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H43" t="n">
-        <v>0.06308900000000001</v>
+        <v>0.082693</v>
       </c>
     </row>
     <row r="44">
@@ -1991,34 +1991,34 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>spectral_centroid</t>
+          <t>peak_last_pos</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>6.1379e-02</t>
+          <t>7.6832e-02</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>6.0737e-03</t>
+          <t>1.6614e-03</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>1.8569e-01</t>
+          <t>-7.9049e-02</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>5.9798e-17</t>
+          <t>1.2124e-03</t>
         </is>
       </c>
       <c r="G44" t="n">
-        <v>1997</v>
+        <v>1673</v>
       </c>
       <c r="H44" t="n">
-        <v>0.061379</v>
+        <v>0.076832</v>
       </c>
     </row>
     <row r="45">
@@ -2027,34 +2027,34 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>spectral_spread</t>
+          <t>peak_first_pos</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>5.9047e-02</t>
+          <t>7.4971e-02</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>8.3073e-03</t>
+          <t>2.1513e-03</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>8.8731e-02</t>
+          <t>7.5897e-02</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>7.1703e-05</t>
+          <t>1.8930e-03</t>
         </is>
       </c>
       <c r="G45" t="n">
-        <v>1997</v>
+        <v>1673</v>
       </c>
       <c r="H45" t="n">
-        <v>0.059047</v>
+        <v>0.074971</v>
       </c>
     </row>
     <row r="46">
@@ -2063,34 +2063,34 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>wavelet_cD3_energy</t>
+          <t>spectral_spread</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>5.3477e-02</t>
+          <t>7.1770e-02</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>1.6125e-02</t>
+          <t>3.3124e-03</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>2.2470e-02</t>
+          <t>7.2485e-02</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>3.1231e-01</t>
+          <t>3.0121e-03</t>
         </is>
       </c>
       <c r="G46" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H46" t="n">
-        <v>0.053477</v>
+        <v>0.07177</v>
       </c>
     </row>
     <row r="47">
@@ -2099,34 +2099,34 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>fft_mag_mean</t>
+          <t>slope_max</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>-5.2876e-02</t>
+          <t>6.5633e-02</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>1.7359e-02</t>
+          <t>7.2438e-03</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>-5.9406e-02</t>
+          <t>7.4768e-02</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>7.5104e-03</t>
+          <t>2.2121e-03</t>
         </is>
       </c>
       <c r="G47" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H47" t="n">
-        <v>0.052876</v>
+        <v>0.065633</v>
       </c>
     </row>
     <row r="48">
@@ -2135,34 +2135,34 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>wavelet_cD2_energy</t>
+          <t>wavelet_cD3_energy</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>5.0171e-02</t>
+          <t>6.4768e-02</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>2.3999e-02</t>
+          <t>8.0496e-03</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>5.2341e-02</t>
+          <t>5.6467e-02</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>1.8526e-02</t>
+          <t>2.0902e-02</t>
         </is>
       </c>
       <c r="G48" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H48" t="n">
-        <v>0.050171</v>
+        <v>0.06476800000000001</v>
       </c>
     </row>
     <row r="49">
@@ -2171,34 +2171,34 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>spectral_rolloff</t>
+          <t>wavelet_cD2_energy</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>5.0114e-02</t>
+          <t>6.4275e-02</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>2.5125e-02</t>
+          <t>8.5448e-03</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>1.6363e-01</t>
+          <t>1.0072e-01</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>1.8762e-13</t>
+          <t>3.6754e-05</t>
         </is>
       </c>
       <c r="G49" t="n">
-        <v>1997</v>
+        <v>1673</v>
       </c>
       <c r="H49" t="n">
-        <v>0.050114</v>
+        <v>0.064275</v>
       </c>
     </row>
     <row r="50">
@@ -2212,29 +2212,29 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>4.8834e-02</t>
+          <t>6.0501e-02</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>2.9094e-02</t>
+          <t>1.3322e-02</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>9.7036e-02</t>
+          <t>8.9659e-02</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>1.3999e-05</t>
+          <t>2.4073e-04</t>
         </is>
       </c>
       <c r="G50" t="n">
-        <v>1997</v>
+        <v>1673</v>
       </c>
       <c r="H50" t="n">
-        <v>0.048834</v>
+        <v>0.060501</v>
       </c>
     </row>
     <row r="51">
@@ -2243,34 +2243,34 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>slope_max</t>
+          <t>band1_energy_ratio</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>4.3166e-02</t>
+          <t>-5.6355e-02</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>5.2172e-02</t>
+          <t>2.1159e-02</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>3.3123e-02</t>
+          <t>-8.7507e-02</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>1.3631e-01</t>
+          <t>3.3908e-04</t>
         </is>
       </c>
       <c r="G51" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H51" t="n">
-        <v>0.043166</v>
+        <v>0.056355</v>
       </c>
     </row>
     <row r="52">
@@ -2279,34 +2279,34 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>range</t>
+          <t>wavelet_cD2_std</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>-3.8558e-02</t>
+          <t>5.5368e-02</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>8.2873e-02</t>
+          <t>2.3530e-02</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>-3.8331e-02</t>
+          <t>6.9322e-02</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>8.4704e-02</t>
+          <t>4.5578e-03</t>
         </is>
       </c>
       <c r="G52" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H52" t="n">
-        <v>0.038558</v>
+        <v>0.055368</v>
       </c>
     </row>
     <row r="53">
@@ -2315,34 +2315,34 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>band1_energy_ratio</t>
+          <t>wavelet_cD3_std</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>-3.5850e-02</t>
+          <t>5.1071e-02</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>1.0925e-01</t>
+          <t>3.6734e-02</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>-9.9387e-02</t>
+          <t>3.7295e-02</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>8.6018e-06</t>
+          <t>1.2730e-01</t>
         </is>
       </c>
       <c r="G53" t="n">
-        <v>1997</v>
+        <v>1673</v>
       </c>
       <c r="H53" t="n">
-        <v>0.03585</v>
+        <v>0.051071</v>
       </c>
     </row>
     <row r="54">
@@ -2351,34 +2351,34 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>wavelet_cD3_std</t>
+          <t>band3_energy_ratio</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>3.2704e-02</t>
+          <t>4.7450e-02</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>1.4135e-01</t>
+          <t>5.2325e-02</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>6.1700e-03</t>
+          <t>8.4469e-02</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>7.8146e-01</t>
+          <t>5.4303e-04</t>
         </is>
       </c>
       <c r="G54" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H54" t="n">
-        <v>0.032704</v>
+        <v>0.04745</v>
       </c>
     </row>
     <row r="55">
@@ -2387,34 +2387,34 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>wavelet_cD2_std</t>
+          <t>band4_energy_ratio</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>3.2248e-02</t>
+          <t>4.6359e-02</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>1.4698e-01</t>
+          <t>5.7985e-02</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>3.2047e-02</t>
+          <t>8.0829e-02</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>1.4952e-01</t>
+          <t>9.3615e-04</t>
         </is>
       </c>
       <c r="G55" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H55" t="n">
-        <v>0.032248</v>
+        <v>0.046359</v>
       </c>
     </row>
     <row r="56">
@@ -2423,34 +2423,34 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>peak_count</t>
+          <t>fft_mag_mean</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2.9972e-02</t>
+          <t>-4.3813e-02</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>1.7770e-01</t>
+          <t>7.3202e-02</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>2.6371e-02</t>
+          <t>-3.8694e-02</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>2.3567e-01</t>
+          <t>1.1363e-01</t>
         </is>
       </c>
       <c r="G56" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H56" t="n">
-        <v>0.029972</v>
+        <v>0.043813</v>
       </c>
     </row>
     <row r="57">
@@ -2459,34 +2459,34 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>band1_energy</t>
+          <t>peak_count</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>-2.9023e-02</t>
+          <t>4.2093e-02</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>1.9184e-01</t>
+          <t>8.5217e-02</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>-8.5198e-02</t>
+          <t>5.9871e-02</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>1.2425e-04</t>
+          <t>1.4317e-02</t>
         </is>
       </c>
       <c r="G57" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H57" t="n">
-        <v>0.029023</v>
+        <v>0.042093</v>
       </c>
     </row>
     <row r="58">
@@ -2495,34 +2495,34 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>spectral_energy</t>
+          <t>slope_abs_mean</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>-2.8875e-02</t>
+          <t>4.1828e-02</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>1.9410e-01</t>
+          <t>8.7201e-02</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>-8.4014e-02</t>
+          <t>7.7314e-02</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>1.5430e-04</t>
+          <t>1.5524e-03</t>
         </is>
       </c>
       <c r="G58" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H58" t="n">
-        <v>0.028875</v>
+        <v>0.041828</v>
       </c>
     </row>
     <row r="59">
@@ -2531,34 +2531,34 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>band3_energy_ratio</t>
+          <t>wavelet_cD1_std</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2.4433e-02</t>
+          <t>4.0293e-02</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>2.7513e-01</t>
+          <t>9.9449e-02</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>9.6721e-02</t>
+          <t>4.3124e-02</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>1.4930e-05</t>
+          <t>7.7840e-02</t>
         </is>
       </c>
       <c r="G59" t="n">
-        <v>1997</v>
+        <v>1673</v>
       </c>
       <c r="H59" t="n">
-        <v>0.024433</v>
+        <v>0.040293</v>
       </c>
     </row>
     <row r="60">
@@ -2567,34 +2567,34 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>wavelet_cD1_std</t>
+          <t>range</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>1.7552e-02</t>
+          <t>-2.5167e-02</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>4.2998e-01</t>
+          <t>3.0359e-01</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>4.4375e-03</t>
+          <t>-9.5018e-03</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>8.4186e-01</t>
+          <t>6.9775e-01</t>
         </is>
       </c>
       <c r="G60" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H60" t="n">
-        <v>0.017552</v>
+        <v>0.025167</v>
       </c>
     </row>
     <row r="61">
@@ -2603,34 +2603,34 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>band4_energy_ratio</t>
+          <t>band1_energy</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>1.7218e-02</t>
+          <t>-1.9752e-02</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>4.4188e-01</t>
+          <t>4.1944e-01</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>9.5545e-02</t>
+          <t>-7.5983e-02</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>1.8958e-05</t>
+          <t>1.8705e-03</t>
         </is>
       </c>
       <c r="G61" t="n">
-        <v>1997</v>
+        <v>1673</v>
       </c>
       <c r="H61" t="n">
-        <v>0.017218</v>
+        <v>0.019752</v>
       </c>
     </row>
     <row r="62">
@@ -2639,34 +2639,34 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>slope_abs_mean</t>
+          <t>spectral_energy</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>1.1479e-02</t>
+          <t>-1.9441e-02</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>6.0578e-01</t>
+          <t>4.2681e-01</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2.9837e-02</t>
+          <t>-7.4475e-02</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>1.7966e-01</t>
+          <t>2.3025e-03</t>
         </is>
       </c>
       <c r="G62" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H62" t="n">
-        <v>0.011479</v>
+        <v>0.019441</v>
       </c>
     </row>
     <row r="63">
@@ -2675,34 +2675,34 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>wavelet_energy_ratio_D1</t>
+          <t>band4_energy</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>-1.0734e-02</t>
+          <t>1.1960e-02</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>6.2935e-01</t>
+          <t>6.2496e-01</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>-7.2749e-02</t>
+          <t>-1.6721e-02</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>1.0558e-03</t>
+          <t>4.9432e-01</t>
         </is>
       </c>
       <c r="G63" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H63" t="n">
-        <v>0.010734</v>
+        <v>0.01196</v>
       </c>
     </row>
     <row r="64">
@@ -2711,34 +2711,34 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>band2_energy</t>
+          <t>band3_energy</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>-8.7722e-03</t>
+          <t>1.1306e-02</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>6.9328e-01</t>
+          <t>6.4401e-01</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>-4.3109e-02</t>
+          <t>-1.6545e-02</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>5.2485e-02</t>
+          <t>4.9887e-01</t>
         </is>
       </c>
       <c r="G64" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H64" t="n">
-        <v>0.008772200000000001</v>
+        <v>0.011306</v>
       </c>
     </row>
     <row r="65">
@@ -2747,34 +2747,34 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>band3_energy</t>
+          <t>band2_energy</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>-7.7725e-03</t>
+          <t>9.9913e-03</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>7.2674e-01</t>
+          <t>6.8300e-01</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>-4.2855e-02</t>
+          <t>-1.7675e-02</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>5.3890e-02</t>
+          <t>4.7000e-01</t>
         </is>
       </c>
       <c r="G65" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H65" t="n">
-        <v>0.0077725</v>
+        <v>0.0099913</v>
       </c>
     </row>
     <row r="66">
@@ -2783,34 +2783,34 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>band4_energy</t>
+          <t>wavelet_energy_ratio_D1</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>-7.3534e-03</t>
+          <t>-5.8013e-03</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>7.4093e-01</t>
+          <t>8.1257e-01</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>-4.2459e-02</t>
+          <t>-6.5978e-02</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>5.6150e-02</t>
+          <t>6.9426e-03</t>
         </is>
       </c>
       <c r="G66" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H66" t="n">
-        <v>0.0073534</v>
+        <v>0.0058013</v>
       </c>
     </row>
   </sheetData>
@@ -2875,34 +2875,34 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>skewness</t>
+          <t>p25</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>-3.3129e-01</t>
+          <t>3.6644e-01</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>8.6009e-46</t>
+          <t>2.5306e-54</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>-3.3399e-01</t>
+          <t>3.6956e-01</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1.4808e-46</t>
+          <t>2.7359e-55</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>1738</v>
+        <v>1673</v>
       </c>
       <c r="H2" t="n">
-        <v>0.33129</v>
+        <v>0.36644</v>
       </c>
     </row>
     <row r="3">
@@ -2911,34 +2911,34 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>p25</t>
+          <t>p10</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>3.0930e-01</t>
+          <t>3.5776e-01</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>4.0245e-46</t>
+          <t>1.0943e-51</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>3.1692e-01</t>
+          <t>3.5255e-01</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>1.8684e-48</t>
+          <t>3.8373e-50</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H3" t="n">
-        <v>0.3093</v>
+        <v>0.35776</v>
       </c>
     </row>
     <row r="4">
@@ -2947,34 +2947,34 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>p10</t>
+          <t>CV</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3.0799e-01</t>
+          <t>-3.4903e-01</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>9.9720e-46</t>
+          <t>4.0679e-49</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>3.1347e-01</t>
+          <t>-3.5984e-01</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2.1750e-47</t>
+          <t>2.5995e-52</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H4" t="n">
-        <v>0.30799</v>
+        <v>0.34903</v>
       </c>
     </row>
     <row r="5">
@@ -2988,29 +2988,29 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3.0341e-01</t>
+          <t>3.4342e-01</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2.2993e-44</t>
+          <t>1.6487e-47</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2.7255e-01</t>
+          <t>3.2372e-01</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>8.3381e-36</t>
+          <t>4.0805e-42</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H5" t="n">
-        <v>0.30341</v>
+        <v>0.34342</v>
       </c>
     </row>
     <row r="6">
@@ -3019,34 +3019,34 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>AUC</t>
+          <t>skewness</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2.9834e-01</t>
+          <t>-3.4332e-01</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6.9312e-43</t>
+          <t>1.7578e-47</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>3.0392e-01</t>
+          <t>-3.2715e-01</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>1.6227e-44</t>
+          <t>5.0009e-43</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H6" t="n">
-        <v>0.29834</v>
+        <v>0.34332</v>
       </c>
     </row>
     <row r="7">
@@ -3055,34 +3055,34 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>peak_mean_height</t>
+          <t>kurtosis</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2.9743e-01</t>
+          <t>3.3102e-01</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1.6018e-35</t>
+          <t>4.5303e-44</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>3.2378e-01</t>
+          <t>3.8909e-01</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>3.9207e-42</t>
+          <t>1.3591e-61</t>
         </is>
       </c>
       <c r="G7" t="n">
         <v>1673</v>
       </c>
       <c r="H7" t="n">
-        <v>0.29743</v>
+        <v>0.33102</v>
       </c>
     </row>
     <row r="8">
@@ -3091,34 +3091,34 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>wavelet_cA_energy</t>
+          <t>AUC</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2.8136e-01</t>
+          <t>3.3086e-01</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.8634e-38</t>
+          <t>5.0127e-44</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2.4854e-01</t>
+          <t>3.4466e-01</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>7.1358e-30</t>
+          <t>7.3014e-48</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H8" t="n">
-        <v>0.28136</v>
+        <v>0.33086</v>
       </c>
     </row>
     <row r="9">
@@ -3127,34 +3127,34 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>kurtosis</t>
+          <t>median</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2.7751e-01</t>
+          <t>3.2903e-01</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>4.2214e-32</t>
+          <t>1.5664e-43</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3.9515e-01</t>
+          <t>3.3747e-01</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>4.8330e-66</t>
+          <t>7.7459e-46</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>1738</v>
+        <v>1673</v>
       </c>
       <c r="H9" t="n">
-        <v>0.27751</v>
+        <v>0.32903</v>
       </c>
     </row>
     <row r="10">
@@ -3163,34 +3163,34 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>p5</t>
+          <t>wavelet_cA_energy</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2.7029e-01</t>
+          <t>3.2281e-01</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>3.1972e-35</t>
+          <t>7.0719e-42</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2.7232e-01</t>
+          <t>2.9972e-01</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>9.5299e-36</t>
+          <t>4.5505e-36</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H10" t="n">
-        <v>0.27029</v>
+        <v>0.32281</v>
       </c>
     </row>
     <row r="11">
@@ -3199,34 +3199,34 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>median</t>
+          <t>p90_p10_ratio</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2.6759e-01</t>
+          <t>-3.1834e-01</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1.5694e-34</t>
+          <t>1.0327e-40</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2.7686e-01</t>
+          <t>-3.5191e-01</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>6.1348e-37</t>
+          <t>5.9040e-50</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H11" t="n">
-        <v>0.26759</v>
+        <v>0.31834</v>
       </c>
     </row>
     <row r="12">
@@ -3235,34 +3235,34 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>min</t>
+          <t>p5</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2.6597e-01</t>
+          <t>3.0393e-01</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>4.0645e-34</t>
+          <t>4.3413e-37</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2.7455e-01</t>
+          <t>2.9402e-01</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2.4949e-36</t>
+          <t>1.0259e-34</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H12" t="n">
-        <v>0.26597</v>
+        <v>0.30393</v>
       </c>
     </row>
     <row r="13">
@@ -3271,34 +3271,34 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>p90_p10_ratio</t>
+          <t>min</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>-2.6350e-01</t>
+          <t>2.9746e-01</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>1.6941e-33</t>
+          <t>1.5763e-35</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>-2.8949e-01</t>
+          <t>2.9885e-01</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2.2689e-40</t>
+          <t>7.3495e-36</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H13" t="n">
-        <v>0.2635</v>
+        <v>0.29746</v>
       </c>
     </row>
     <row r="14">
@@ -3307,34 +3307,34 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>peak_max_width</t>
+          <t>peak_mean_height</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2.6156e-01</t>
+          <t>2.9743e-01</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>1.4288e-27</t>
+          <t>1.6018e-35</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>3.0469e-01</t>
+          <t>3.2378e-01</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2.8193e-37</t>
+          <t>3.9207e-42</t>
         </is>
       </c>
       <c r="G14" t="n">
         <v>1673</v>
       </c>
       <c r="H14" t="n">
-        <v>0.26156</v>
+        <v>0.29743</v>
       </c>
     </row>
     <row r="15">
@@ -3343,34 +3343,34 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CV</t>
+          <t>AUC_normalized</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>-2.5882e-01</t>
+          <t>2.9738e-01</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2.4535e-32</t>
+          <t>1.6476e-35</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>-2.9598e-01</t>
+          <t>3.0680e-01</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>3.3202e-42</t>
+          <t>8.5343e-38</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H15" t="n">
-        <v>0.25882</v>
+        <v>0.29738</v>
       </c>
     </row>
     <row r="16">
@@ -3379,34 +3379,34 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>peak_max_height</t>
+          <t>mean</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2.4627e-01</t>
+          <t>2.9683e-01</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>1.5613e-24</t>
+          <t>2.2272e-35</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2.7520e-01</t>
+          <t>3.0620e-01</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>1.8682e-30</t>
+          <t>1.1995e-37</t>
         </is>
       </c>
       <c r="G16" t="n">
         <v>1673</v>
       </c>
       <c r="H16" t="n">
-        <v>0.24627</v>
+        <v>0.29683</v>
       </c>
     </row>
     <row r="17">
@@ -3415,34 +3415,34 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>AUC_normalized</t>
+          <t>IQR</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2.3893e-01</t>
+          <t>-2.6372e-01</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1.1413e-27</t>
+          <t>5.1269e-28</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2.5128e-01</t>
+          <t>-2.8742e-01</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>1.6169e-30</t>
+          <t>3.4962e-33</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H17" t="n">
-        <v>0.23893</v>
+        <v>0.26372</v>
       </c>
     </row>
     <row r="18">
@@ -3451,34 +3451,34 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>mean</t>
+          <t>peak_max_width</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2.3835e-01</t>
+          <t>2.6156e-01</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>1.5393e-27</t>
+          <t>1.4288e-27</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2.4982e-01</t>
+          <t>3.0469e-01</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>3.5831e-30</t>
+          <t>2.8193e-37</t>
         </is>
       </c>
       <c r="G18" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H18" t="n">
-        <v>0.23835</v>
+        <v>0.26156</v>
       </c>
     </row>
     <row r="19">
@@ -3487,34 +3487,34 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>peak_mean_width</t>
+          <t>peak_max_height</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2.3665e-01</t>
+          <t>2.4627e-01</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1.0010e-22</t>
+          <t>1.5613e-24</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2.4913e-01</t>
+          <t>2.7520e-01</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>4.3631e-25</t>
+          <t>1.8682e-30</t>
         </is>
       </c>
       <c r="G19" t="n">
         <v>1673</v>
       </c>
       <c r="H19" t="n">
-        <v>0.23665</v>
+        <v>0.24627</v>
       </c>
     </row>
     <row r="20">
@@ -3523,34 +3523,34 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>IQR</t>
+          <t>dominant_freq</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>-2.2228e-01</t>
+          <t>2.4549e-01</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>4.4729e-24</t>
+          <t>2.1957e-24</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>-2.4286e-01</t>
+          <t>1.9218e-01</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>1.4700e-28</t>
+          <t>2.2173e-15</t>
         </is>
       </c>
       <c r="G20" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H20" t="n">
-        <v>0.22228</v>
+        <v>0.24549</v>
       </c>
     </row>
     <row r="21">
@@ -3559,34 +3559,34 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>signal_length</t>
+          <t>peak_mean_width</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>1.9536e-01</t>
+          <t>2.3665e-01</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>7.3748e-19</t>
+          <t>1.0010e-22</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2.4338e-01</t>
+          <t>2.4913e-01</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>1.1199e-28</t>
+          <t>4.3631e-25</t>
         </is>
       </c>
       <c r="G21" t="n">
-        <v>2024</v>
+        <v>1673</v>
       </c>
       <c r="H21" t="n">
-        <v>0.19536</v>
+        <v>0.23665</v>
       </c>
     </row>
   </sheetData>
@@ -3622,7 +3622,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>74.396</v>
+        <v>72.17700000000001</v>
       </c>
     </row>
     <row r="3">
@@ -3632,7 +3632,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>59.312</v>
+        <v>58.252</v>
       </c>
     </row>
     <row r="4">
@@ -3642,7 +3642,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3.612</v>
+        <v>3.567</v>
       </c>
     </row>
     <row r="5">
@@ -3652,7 +3652,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2.39</v>
+        <v>2.351</v>
       </c>
     </row>
     <row r="6">
@@ -3662,7 +3662,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1.404</v>
+        <v>1.445</v>
       </c>
     </row>
     <row r="7">
@@ -3672,7 +3672,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1.273</v>
+        <v>1.268</v>
       </c>
     </row>
     <row r="8">
@@ -3682,7 +3682,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1.148</v>
+        <v>1.149</v>
       </c>
     </row>
   </sheetData>
@@ -3763,22 +3763,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>820</v>
+        <v>665</v>
       </c>
       <c r="C2" t="n">
-        <v>148.81</v>
+        <v>149.52</v>
       </c>
       <c r="D2" t="n">
-        <v>28.04</v>
+        <v>27.46</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="F2" t="n">
         <v>132</v>
       </c>
       <c r="G2" t="n">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H2" t="n">
         <v>166</v>
@@ -3790,7 +3790,7 @@
         <v>118</v>
       </c>
       <c r="K2" t="n">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="3">
@@ -3800,16 +3800,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1204</v>
+        <v>1008</v>
       </c>
       <c r="C3" t="n">
-        <v>104.75</v>
+        <v>104.69</v>
       </c>
       <c r="D3" t="n">
-        <v>16.19</v>
+        <v>15.71</v>
       </c>
       <c r="E3" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="F3" t="n">
         <v>95</v>
@@ -3818,7 +3818,7 @@
         <v>103</v>
       </c>
       <c r="H3" t="n">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I3" t="n">
         <v>190</v>

</xml_diff>